<commit_message>
correction in data mdel
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7D1C03-8286-422C-B905-9973506317F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB20B52A-ADCD-4935-AA1F-35730C95448C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="13" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18687" uniqueCount="4706">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18654" uniqueCount="4698">
   <si>
     <t>Domain</t>
   </si>
@@ -13642,9 +13642,6 @@
     <t>REL091</t>
   </si>
   <si>
-    <t>Each QR Scan History record has one scan result classification.</t>
-  </si>
-  <si>
     <t>REL092</t>
   </si>
   <si>
@@ -13915,31 +13912,10 @@
     <t>Identifies the membership product acquired through the QR journey.</t>
   </si>
   <si>
-    <t>QR Code has Scan History</t>
-  </si>
-  <si>
-    <t>Each QR scan history record references the QR Code that was scanned.</t>
-  </si>
-  <si>
-    <t>QR Code has QR Code Type</t>
-  </si>
-  <si>
-    <t>Identifies the journey type configured for the QR Code.</t>
-  </si>
-  <si>
     <t>REL095</t>
   </si>
   <si>
     <t>REL096</t>
-  </si>
-  <si>
-    <t>REL097</t>
-  </si>
-  <si>
-    <t>REL098</t>
-  </si>
-  <si>
-    <t>REL099</t>
   </si>
   <si>
     <t>CXREL</t>
@@ -16703,7 +16679,7 @@
     </row>
     <row r="38" spans="1:17" ht="105">
       <c r="A38" s="4" t="s">
-        <v>4699</v>
+        <v>4691</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>2333</v>
@@ -17427,22 +17403,22 @@
     </row>
     <row r="52" spans="1:17" ht="60">
       <c r="A52" s="4" t="s">
-        <v>4579</v>
+        <v>4578</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>731</v>
       </c>
       <c r="C52" s="4" t="s">
+        <v>4579</v>
+      </c>
+      <c r="D52" s="4" t="s">
         <v>4580</v>
       </c>
-      <c r="D52" s="4" t="s">
+      <c r="E52" s="4" t="s">
         <v>4581</v>
       </c>
-      <c r="E52" s="4" t="s">
+      <c r="F52" s="4" t="s">
         <v>4582</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>4583</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>621</v>
@@ -17466,39 +17442,39 @@
         <v>7</v>
       </c>
       <c r="N52" s="4" t="s">
+        <v>4583</v>
+      </c>
+      <c r="O52" s="4" t="s">
         <v>4584</v>
-      </c>
-      <c r="O52" s="4" t="s">
-        <v>4585</v>
       </c>
       <c r="P52" s="4" t="s">
         <v>46</v>
       </c>
       <c r="Q52" s="4" t="s">
-        <v>4586</v>
+        <v>4585</v>
       </c>
     </row>
     <row r="53" spans="1:17" ht="105">
       <c r="A53" s="4" t="s">
-        <v>4632</v>
+        <v>4624</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>2333</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>4633</v>
+        <v>4625</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>4635</v>
+        <v>4627</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>4636</v>
+        <v>4628</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>4637</v>
+        <v>4629</v>
       </c>
       <c r="H53" s="4" t="s">
         <v>261</v>
@@ -17519,16 +17495,16 @@
         <v>7</v>
       </c>
       <c r="N53" s="4" t="s">
-        <v>4638</v>
+        <v>4630</v>
       </c>
       <c r="O53" s="4" t="s">
-        <v>4639</v>
+        <v>4631</v>
       </c>
       <c r="P53" s="4" t="s">
-        <v>4640</v>
+        <v>4632</v>
       </c>
       <c r="Q53" s="4" t="s">
-        <v>4641</v>
+        <v>4633</v>
       </c>
     </row>
   </sheetData>
@@ -19409,7 +19385,7 @@
         <v>4379</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>4578</v>
+        <v>4577</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>2218</v>
@@ -21106,7 +21082,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
-  <dimension ref="A1:K99"/>
+  <dimension ref="A1:K96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
@@ -22088,7 +22064,7 @@
         <v>263</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>4704</v>
+        <v>4696</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>7</v>
@@ -22683,7 +22659,7 @@
         <v>23</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>4704</v>
+        <v>4696</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>7</v>
@@ -22718,7 +22694,7 @@
         <v>23</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>4704</v>
+        <v>4696</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>7</v>
@@ -22788,7 +22764,7 @@
         <v>23</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>4704</v>
+        <v>4696</v>
       </c>
       <c r="H48" s="3" t="s">
         <v>7</v>
@@ -23889,7 +23865,7 @@
       </c>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="4" t="s">
+      <c r="A80" s="3" t="s">
         <v>4371</v>
       </c>
       <c r="B80" s="4" t="s">
@@ -23924,7 +23900,7 @@
       </c>
     </row>
     <row r="81" spans="1:11">
-      <c r="A81" s="4" t="s">
+      <c r="A81" s="3" t="s">
         <v>4373</v>
       </c>
       <c r="B81" s="4" t="s">
@@ -23959,7 +23935,7 @@
       </c>
     </row>
     <row r="82" spans="1:11">
-      <c r="A82" s="4" t="s">
+      <c r="A82" s="3" t="s">
         <v>4375</v>
       </c>
       <c r="B82" s="4" t="s">
@@ -23994,7 +23970,7 @@
       </c>
     </row>
     <row r="83" spans="1:11">
-      <c r="A83" s="4" t="s">
+      <c r="A83" s="3" t="s">
         <v>4509</v>
       </c>
       <c r="B83" s="4" t="s">
@@ -24029,7 +24005,7 @@
       </c>
     </row>
     <row r="84" spans="1:11">
-      <c r="A84" s="4" t="s">
+      <c r="A84" s="3" t="s">
         <v>4510</v>
       </c>
       <c r="B84" s="4" t="s">
@@ -24064,7 +24040,7 @@
       </c>
     </row>
     <row r="85" spans="1:11" ht="30">
-      <c r="A85" s="4" t="s">
+      <c r="A85" s="3" t="s">
         <v>4513</v>
       </c>
       <c r="B85" s="4" t="s">
@@ -24099,7 +24075,7 @@
       </c>
     </row>
     <row r="86" spans="1:11">
-      <c r="A86" s="4" t="s">
+      <c r="A86" s="3" t="s">
         <v>4516</v>
       </c>
       <c r="B86" s="4" t="s">
@@ -24134,7 +24110,7 @@
       </c>
     </row>
     <row r="87" spans="1:11">
-      <c r="A87" s="4" t="s">
+      <c r="A87" s="3" t="s">
         <v>4519</v>
       </c>
       <c r="B87" s="4" t="s">
@@ -24169,7 +24145,7 @@
       </c>
     </row>
     <row r="88" spans="1:11">
-      <c r="A88" s="4" t="s">
+      <c r="A88" s="3" t="s">
         <v>4522</v>
       </c>
       <c r="B88" s="4" t="s">
@@ -24204,7 +24180,7 @@
       </c>
     </row>
     <row r="89" spans="1:11" ht="30">
-      <c r="A89" s="4" t="s">
+      <c r="A89" s="3" t="s">
         <v>4525</v>
       </c>
       <c r="B89" s="4" t="s">
@@ -24238,30 +24214,30 @@
         <v>4530</v>
       </c>
     </row>
-    <row r="90" spans="1:11">
-      <c r="A90" s="4" t="s">
+    <row r="90" spans="1:11" ht="30">
+      <c r="A90" s="3" t="s">
         <v>4528</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>4400</v>
+        <v>34</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>4386</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>4400</v>
+        <v>4533</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>4403</v>
+        <v>692</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>4403</v>
+        <v>692</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>1292</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I90" s="4" t="s">
         <v>175</v>
@@ -24270,27 +24246,27 @@
         <v>6</v>
       </c>
       <c r="K90" s="4" t="s">
-        <v>4532</v>
+        <v>4534</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="30">
-      <c r="A91" s="4" t="s">
+      <c r="A91" s="3" t="s">
         <v>4531</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>4386</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>4534</v>
+        <v>4536</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>1292</v>
@@ -24305,27 +24281,27 @@
         <v>6</v>
       </c>
       <c r="K91" s="4" t="s">
-        <v>4535</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="30">
-      <c r="A92" s="4" t="s">
-        <v>4533</v>
+      <c r="A92" s="3" t="s">
+        <v>4532</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>4386</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>4537</v>
+        <v>4539</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>696</v>
+        <v>51</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>696</v>
+        <v>138</v>
       </c>
       <c r="G92" s="4" t="s">
         <v>1292</v>
@@ -24334,74 +24310,74 @@
         <v>6</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>175</v>
+        <v>4337</v>
       </c>
       <c r="J92" s="4" t="s">
         <v>6</v>
       </c>
       <c r="K92" s="4" t="s">
-        <v>4538</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" ht="30">
-      <c r="A93" s="4" t="s">
-        <v>4536</v>
+        <v>4540</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" ht="45">
+      <c r="A93" s="3" t="s">
+        <v>4535</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>4386</v>
+        <v>4580</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>4540</v>
+        <v>4613</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>138</v>
+        <v>23</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>1292</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>4337</v>
+        <v>175</v>
       </c>
       <c r="J93" s="4" t="s">
         <v>6</v>
       </c>
       <c r="K93" s="4" t="s">
-        <v>4541</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" ht="45">
-      <c r="A94" s="4" t="s">
-        <v>4539</v>
+        <v>4614</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" ht="30">
+      <c r="A94" s="3" t="s">
+        <v>4538</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>5</v>
+        <v>4386</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>4614</v>
+        <v>4615</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>23</v>
+        <v>4389</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>23</v>
+        <v>4389</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>1292</v>
+        <v>4616</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I94" s="4" t="s">
         <v>175</v>
@@ -24410,30 +24386,30 @@
         <v>6</v>
       </c>
       <c r="K94" s="4" t="s">
-        <v>4615</v>
+        <v>4617</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="30">
-      <c r="A95" s="4" t="s">
-        <v>4627</v>
+      <c r="A95" s="3" t="s">
+        <v>4622</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>4386</v>
+        <v>618</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="D95" s="4" t="s">
+        <v>4618</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="G95" s="4" t="s">
         <v>4616</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>4389</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>4389</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>4617</v>
       </c>
       <c r="H95" s="4" t="s">
         <v>6</v>
@@ -24445,33 +24421,33 @@
         <v>6</v>
       </c>
       <c r="K95" s="4" t="s">
-        <v>4618</v>
+        <v>4619</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="30">
-      <c r="A96" s="4" t="s">
-        <v>4628</v>
+      <c r="A96" s="3" t="s">
+        <v>4623</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>618</v>
+        <v>10</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>4619</v>
+        <v>4620</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>622</v>
+        <v>418</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>622</v>
+        <v>418</v>
       </c>
       <c r="G96" s="4" t="s">
-        <v>4617</v>
+        <v>1292</v>
       </c>
       <c r="H96" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>175</v>
@@ -24480,112 +24456,7 @@
         <v>6</v>
       </c>
       <c r="K96" s="4" t="s">
-        <v>4620</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" ht="30">
-      <c r="A97" s="4" t="s">
-        <v>4629</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C97" s="4" t="s">
-        <v>4581</v>
-      </c>
-      <c r="D97" s="4" t="s">
         <v>4621</v>
-      </c>
-      <c r="E97" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="F97" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="G97" s="4" t="s">
-        <v>1292</v>
-      </c>
-      <c r="H97" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I97" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="J97" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="K97" s="4" t="s">
-        <v>4622</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" ht="30">
-      <c r="A98" s="4" t="s">
-        <v>4630</v>
-      </c>
-      <c r="B98" s="4" t="s">
-        <v>4379</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>4386</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>4623</v>
-      </c>
-      <c r="E98" s="4" t="s">
-        <v>4382</v>
-      </c>
-      <c r="F98" s="4" t="s">
-        <v>4382</v>
-      </c>
-      <c r="G98" s="4" t="s">
-        <v>1292</v>
-      </c>
-      <c r="H98" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I98" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="J98" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="K98" s="4" t="s">
-        <v>4624</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11">
-      <c r="A99" s="4" t="s">
-        <v>4631</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>4393</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>4379</v>
-      </c>
-      <c r="D99" s="4" t="s">
-        <v>4625</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>4396</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>4396</v>
-      </c>
-      <c r="G99" s="4" t="s">
-        <v>1292</v>
-      </c>
-      <c r="H99" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I99" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="J99" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="K99" s="4" t="s">
-        <v>4626</v>
       </c>
     </row>
   </sheetData>
@@ -24708,7 +24579,7 @@
         <v>1377</v>
       </c>
       <c r="F4" t="s">
-        <v>4701</v>
+        <v>4693</v>
       </c>
       <c r="G4" t="s">
         <v>1379</v>
@@ -24734,7 +24605,7 @@
         <v>1389</v>
       </c>
       <c r="F5" t="s">
-        <v>4705</v>
+        <v>4697</v>
       </c>
       <c r="G5" t="s">
         <v>1379</v>
@@ -25410,7 +25281,7 @@
         <v>2177</v>
       </c>
       <c r="F31" t="s">
-        <v>4702</v>
+        <v>4694</v>
       </c>
       <c r="G31" t="s">
         <v>1379</v>
@@ -25419,7 +25290,7 @@
         <v>1380</v>
       </c>
       <c r="I31" t="s">
-        <v>4703</v>
+        <v>4695</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -28802,10 +28673,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>4692</v>
+        <v>4684</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>4693</v>
+        <v>4685</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>168</v>
@@ -28823,28 +28694,28 @@
         <v>7</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="L5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>4647</v>
+        <v>4639</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>4694</v>
+        <v>4686</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>4695</v>
+        <v>4687</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>4696</v>
+        <v>4688</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>4697</v>
+        <v>4689</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>4698</v>
+        <v>4690</v>
       </c>
       <c r="S5" s="4" t="s">
         <v>6</v>
@@ -66501,7 +66372,7 @@
         <v>4314</v>
       </c>
       <c r="O551" s="4" t="s">
-        <v>4700</v>
+        <v>4692</v>
       </c>
       <c r="P551" s="4" t="s">
         <v>4316</v>
@@ -69157,16 +69028,16 @@
     </row>
     <row r="589" spans="1:23" ht="45">
       <c r="A589" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B589" s="4">
         <v>1</v>
       </c>
       <c r="C589" s="4" t="s">
-        <v>4587</v>
+        <v>4586</v>
       </c>
       <c r="D589" s="4" t="s">
-        <v>4584</v>
+        <v>4583</v>
       </c>
       <c r="E589" s="4" t="s">
         <v>168</v>
@@ -69196,13 +69067,13 @@
         <v>7</v>
       </c>
       <c r="N589" s="4" t="s">
+        <v>4587</v>
+      </c>
+      <c r="O589" s="4" t="s">
         <v>4588</v>
       </c>
-      <c r="O589" s="4" t="s">
+      <c r="P589" s="4" t="s">
         <v>4589</v>
-      </c>
-      <c r="P589" s="4" t="s">
-        <v>4590</v>
       </c>
       <c r="Q589" s="4" t="s">
         <v>266</v>
@@ -69228,7 +69099,7 @@
     </row>
     <row r="590" spans="1:23" ht="45">
       <c r="A590" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B590" s="4">
         <v>2</v>
@@ -69267,13 +69138,13 @@
         <v>6</v>
       </c>
       <c r="N590" s="4" t="s">
+        <v>4590</v>
+      </c>
+      <c r="O590" s="4" t="s">
         <v>4591</v>
       </c>
-      <c r="O590" s="4" t="s">
+      <c r="P590" s="4" t="s">
         <v>4592</v>
-      </c>
-      <c r="P590" s="4" t="s">
-        <v>4593</v>
       </c>
       <c r="Q590" s="4" t="s">
         <v>266</v>
@@ -69299,7 +69170,7 @@
     </row>
     <row r="591" spans="1:23" ht="45">
       <c r="A591" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B591" s="4">
         <v>3</v>
@@ -69338,13 +69209,13 @@
         <v>6</v>
       </c>
       <c r="N591" s="4" t="s">
+        <v>4593</v>
+      </c>
+      <c r="O591" s="4" t="s">
         <v>4594</v>
       </c>
-      <c r="O591" s="4" t="s">
+      <c r="P591" s="4" t="s">
         <v>4595</v>
-      </c>
-      <c r="P591" s="4" t="s">
-        <v>4596</v>
       </c>
       <c r="Q591" s="4" t="s">
         <v>266</v>
@@ -69370,7 +69241,7 @@
     </row>
     <row r="592" spans="1:23" ht="30">
       <c r="A592" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B592" s="4">
         <v>4</v>
@@ -69409,13 +69280,13 @@
         <v>6</v>
       </c>
       <c r="N592" s="4" t="s">
+        <v>4596</v>
+      </c>
+      <c r="O592" s="4" t="s">
         <v>4597</v>
       </c>
-      <c r="O592" s="4" t="s">
+      <c r="P592" s="4" t="s">
         <v>4598</v>
-      </c>
-      <c r="P592" s="4" t="s">
-        <v>4599</v>
       </c>
       <c r="Q592" s="4" t="s">
         <v>266</v>
@@ -69441,7 +69312,7 @@
     </row>
     <row r="593" spans="1:23" ht="30">
       <c r="A593" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B593" s="4">
         <v>5</v>
@@ -69480,13 +69351,13 @@
         <v>6</v>
       </c>
       <c r="N593" s="4" t="s">
+        <v>4599</v>
+      </c>
+      <c r="O593" s="4" t="s">
         <v>4600</v>
       </c>
-      <c r="O593" s="4" t="s">
+      <c r="P593" s="4" t="s">
         <v>4601</v>
-      </c>
-      <c r="P593" s="4" t="s">
-        <v>4602</v>
       </c>
       <c r="Q593" s="4" t="s">
         <v>266</v>
@@ -69512,7 +69383,7 @@
     </row>
     <row r="594" spans="1:23" ht="45">
       <c r="A594" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B594" s="4">
         <v>6</v>
@@ -69521,7 +69392,7 @@
         <v>36</v>
       </c>
       <c r="D594" s="4" t="s">
-        <v>4603</v>
+        <v>4602</v>
       </c>
       <c r="E594" s="4" t="s">
         <v>168</v>
@@ -69551,13 +69422,13 @@
         <v>6</v>
       </c>
       <c r="N594" s="4" t="s">
+        <v>4603</v>
+      </c>
+      <c r="O594" s="4" t="s">
         <v>4604</v>
       </c>
-      <c r="O594" s="4" t="s">
+      <c r="P594" s="4" t="s">
         <v>4605</v>
-      </c>
-      <c r="P594" s="4" t="s">
-        <v>4606</v>
       </c>
       <c r="Q594" s="4" t="s">
         <v>266</v>
@@ -69583,16 +69454,16 @@
     </row>
     <row r="595" spans="1:23" ht="30">
       <c r="A595" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B595" s="4">
         <v>7</v>
       </c>
       <c r="C595" s="4" t="s">
-        <v>4585</v>
+        <v>4584</v>
       </c>
       <c r="D595" s="4" t="s">
-        <v>4607</v>
+        <v>4606</v>
       </c>
       <c r="E595" s="4" t="s">
         <v>294</v>
@@ -69622,13 +69493,13 @@
         <v>6</v>
       </c>
       <c r="N595" s="4" t="s">
+        <v>4607</v>
+      </c>
+      <c r="O595" s="4" t="s">
         <v>4608</v>
       </c>
-      <c r="O595" s="4" t="s">
+      <c r="P595" s="4" t="s">
         <v>4609</v>
-      </c>
-      <c r="P595" s="4" t="s">
-        <v>4610</v>
       </c>
       <c r="Q595" s="4" t="s">
         <v>235</v>
@@ -69654,7 +69525,7 @@
     </row>
     <row r="596" spans="1:23" ht="30">
       <c r="A596" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B596" s="4">
         <v>8</v>
@@ -69696,7 +69567,7 @@
         <v>605</v>
       </c>
       <c r="O596" s="4" t="s">
-        <v>4611</v>
+        <v>4610</v>
       </c>
       <c r="P596" s="4" t="s">
         <v>295</v>
@@ -69725,7 +69596,7 @@
     </row>
     <row r="597" spans="1:23" ht="30">
       <c r="A597" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B597" s="4">
         <v>9</v>
@@ -69764,10 +69635,10 @@
         <v>6</v>
       </c>
       <c r="N597" s="4" t="s">
+        <v>4611</v>
+      </c>
+      <c r="O597" s="4" t="s">
         <v>4612</v>
-      </c>
-      <c r="O597" s="4" t="s">
-        <v>4613</v>
       </c>
       <c r="P597" s="4" t="s">
         <v>295</v>
@@ -69796,7 +69667,7 @@
     </row>
     <row r="598" spans="1:23" ht="30">
       <c r="A598" s="4" t="s">
-        <v>4581</v>
+        <v>4580</v>
       </c>
       <c r="B598" s="4">
         <v>10</v>
@@ -69867,16 +69738,16 @@
     </row>
     <row r="599" spans="1:23" ht="30">
       <c r="A599" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B599" s="4">
         <v>1</v>
       </c>
       <c r="C599" s="4" t="s">
-        <v>4642</v>
+        <v>4634</v>
       </c>
       <c r="D599" s="4" t="s">
-        <v>4638</v>
+        <v>4630</v>
       </c>
       <c r="E599" s="4" t="s">
         <v>168</v>
@@ -69900,16 +69771,16 @@
         <v>73</v>
       </c>
       <c r="N599" s="4" t="s">
-        <v>4643</v>
+        <v>4635</v>
       </c>
       <c r="O599" s="4" t="s">
-        <v>4644</v>
+        <v>4636</v>
       </c>
       <c r="P599" s="4" t="s">
-        <v>4645</v>
+        <v>4637</v>
       </c>
       <c r="Q599" s="4" t="s">
-        <v>4646</v>
+        <v>4638</v>
       </c>
       <c r="S599" s="4" t="s">
         <v>6</v>
@@ -69929,7 +69800,7 @@
     </row>
     <row r="600" spans="1:23" ht="30">
       <c r="A600" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B600" s="4">
         <v>2</v>
@@ -69962,16 +69833,16 @@
         <v>6</v>
       </c>
       <c r="M600" s="4" t="s">
-        <v>4647</v>
+        <v>4639</v>
       </c>
       <c r="N600" s="4" t="s">
-        <v>4648</v>
+        <v>4640</v>
       </c>
       <c r="O600" s="4" t="s">
-        <v>4649</v>
+        <v>4641</v>
       </c>
       <c r="P600" s="4" t="s">
-        <v>4650</v>
+        <v>4642</v>
       </c>
       <c r="Q600" s="4">
         <v>1001</v>
@@ -69994,16 +69865,16 @@
     </row>
     <row r="601" spans="1:23" ht="30">
       <c r="A601" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B601" s="4">
         <v>3</v>
       </c>
       <c r="C601" s="4" t="s">
-        <v>4639</v>
+        <v>4631</v>
       </c>
       <c r="D601" s="4" t="s">
-        <v>4651</v>
+        <v>4643</v>
       </c>
       <c r="E601" s="4" t="s">
         <v>172</v>
@@ -70027,13 +69898,13 @@
         <v>73</v>
       </c>
       <c r="N601" s="4" t="s">
-        <v>4652</v>
+        <v>4644</v>
       </c>
       <c r="O601" s="4" t="s">
-        <v>4653</v>
+        <v>4645</v>
       </c>
       <c r="P601" s="4" t="s">
-        <v>4654</v>
+        <v>4646</v>
       </c>
       <c r="Q601" s="4">
         <v>12</v>
@@ -70059,16 +69930,16 @@
     </row>
     <row r="602" spans="1:23" ht="30">
       <c r="A602" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B602" s="4">
         <v>4</v>
       </c>
       <c r="C602" s="4" t="s">
-        <v>4655</v>
+        <v>4647</v>
       </c>
       <c r="D602" s="4" t="s">
-        <v>4656</v>
+        <v>4648</v>
       </c>
       <c r="E602" s="4" t="s">
         <v>168</v>
@@ -70092,19 +69963,19 @@
         <v>6</v>
       </c>
       <c r="M602" s="4" t="s">
-        <v>4647</v>
+        <v>4639</v>
       </c>
       <c r="N602" s="4" t="s">
-        <v>4657</v>
+        <v>4649</v>
       </c>
       <c r="O602" s="4" t="s">
-        <v>4658</v>
+        <v>4650</v>
       </c>
       <c r="P602" s="4" t="s">
-        <v>4659</v>
+        <v>4651</v>
       </c>
       <c r="Q602" s="4" t="s">
-        <v>4660</v>
+        <v>4652</v>
       </c>
       <c r="S602" s="4" t="s">
         <v>6</v>
@@ -70124,19 +69995,19 @@
     </row>
     <row r="603" spans="1:23" ht="45">
       <c r="A603" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B603" s="4">
         <v>5</v>
       </c>
       <c r="C603" s="4" t="s">
-        <v>4661</v>
+        <v>4653</v>
       </c>
       <c r="D603" s="4" t="s">
-        <v>4662</v>
+        <v>4654</v>
       </c>
       <c r="E603" s="4" t="s">
-        <v>4663</v>
+        <v>4655</v>
       </c>
       <c r="G603" s="4" t="s">
         <v>7</v>
@@ -70157,16 +70028,16 @@
         <v>73</v>
       </c>
       <c r="N603" s="4" t="s">
-        <v>4664</v>
+        <v>4656</v>
       </c>
       <c r="O603" s="4" t="s">
-        <v>4665</v>
+        <v>4657</v>
       </c>
       <c r="P603" s="4" t="s">
-        <v>4666</v>
+        <v>4658</v>
       </c>
       <c r="Q603" s="4" t="s">
-        <v>4667</v>
+        <v>4659</v>
       </c>
       <c r="S603" s="4" t="s">
         <v>6</v>
@@ -70186,7 +70057,7 @@
     </row>
     <row r="604" spans="1:23" ht="30">
       <c r="A604" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B604" s="4">
         <v>6</v>
@@ -70219,16 +70090,16 @@
         <v>73</v>
       </c>
       <c r="N604" s="4" t="s">
-        <v>4668</v>
+        <v>4660</v>
       </c>
       <c r="O604" s="4" t="s">
-        <v>4669</v>
+        <v>4661</v>
       </c>
       <c r="P604" s="4" t="s">
-        <v>4670</v>
+        <v>4662</v>
       </c>
       <c r="Q604" s="4" t="s">
-        <v>4671</v>
+        <v>4663</v>
       </c>
       <c r="S604" s="4" t="s">
         <v>6</v>
@@ -70248,7 +70119,7 @@
     </row>
     <row r="605" spans="1:23" ht="30">
       <c r="A605" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B605" s="4">
         <v>7</v>
@@ -70281,16 +70152,16 @@
         <v>6</v>
       </c>
       <c r="M605" s="4" t="s">
-        <v>4647</v>
+        <v>4639</v>
       </c>
       <c r="N605" s="4" t="s">
-        <v>4672</v>
+        <v>4664</v>
       </c>
       <c r="O605" s="4" t="s">
-        <v>4673</v>
+        <v>4665</v>
       </c>
       <c r="P605" s="4" t="s">
-        <v>4674</v>
+        <v>4666</v>
       </c>
       <c r="Q605" s="4" t="s">
         <v>2380</v>
@@ -70313,7 +70184,7 @@
     </row>
     <row r="606" spans="1:23" ht="30">
       <c r="A606" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B606" s="4">
         <v>8</v>
@@ -70346,16 +70217,16 @@
         <v>73</v>
       </c>
       <c r="N606" s="4" t="s">
-        <v>4675</v>
+        <v>4667</v>
       </c>
       <c r="O606" s="4" t="s">
-        <v>4676</v>
+        <v>4668</v>
       </c>
       <c r="P606" s="4" t="s">
-        <v>4677</v>
+        <v>4669</v>
       </c>
       <c r="Q606" s="4" t="s">
-        <v>4671</v>
+        <v>4663</v>
       </c>
       <c r="S606" s="4" t="s">
         <v>6</v>
@@ -70375,7 +70246,7 @@
     </row>
     <row r="607" spans="1:23" ht="30">
       <c r="A607" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B607" s="4">
         <v>9</v>
@@ -70408,16 +70279,16 @@
         <v>6</v>
       </c>
       <c r="M607" s="4" t="s">
-        <v>4647</v>
+        <v>4639</v>
       </c>
       <c r="N607" s="4" t="s">
-        <v>4678</v>
+        <v>4670</v>
       </c>
       <c r="O607" s="4" t="s">
-        <v>4679</v>
+        <v>4671</v>
       </c>
       <c r="P607" s="4" t="s">
-        <v>4680</v>
+        <v>4672</v>
       </c>
       <c r="Q607" s="4" t="s">
         <v>2380</v>
@@ -70440,7 +70311,7 @@
     </row>
     <row r="608" spans="1:23" ht="30">
       <c r="A608" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B608" s="4">
         <v>10</v>
@@ -70473,16 +70344,16 @@
         <v>73</v>
       </c>
       <c r="N608" s="4" t="s">
-        <v>4681</v>
+        <v>4673</v>
       </c>
       <c r="O608" s="4" t="s">
-        <v>4682</v>
+        <v>4674</v>
       </c>
       <c r="P608" s="4" t="s">
-        <v>4683</v>
+        <v>4675</v>
       </c>
       <c r="Q608" s="4" t="s">
-        <v>4671</v>
+        <v>4663</v>
       </c>
       <c r="S608" s="4" t="s">
         <v>6</v>
@@ -70502,7 +70373,7 @@
     </row>
     <row r="609" spans="1:23" ht="30">
       <c r="A609" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B609" s="4">
         <v>11</v>
@@ -70535,16 +70406,16 @@
         <v>6</v>
       </c>
       <c r="M609" s="4" t="s">
-        <v>4647</v>
+        <v>4639</v>
       </c>
       <c r="N609" s="4" t="s">
-        <v>4684</v>
+        <v>4676</v>
       </c>
       <c r="O609" s="4" t="s">
-        <v>4685</v>
+        <v>4677</v>
       </c>
       <c r="P609" s="4" t="s">
-        <v>4686</v>
+        <v>4678</v>
       </c>
       <c r="Q609" s="4" t="s">
         <v>2380</v>
@@ -70567,7 +70438,7 @@
     </row>
     <row r="610" spans="1:23" ht="30">
       <c r="A610" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B610" s="4">
         <v>12</v>
@@ -70603,10 +70474,10 @@
         <v>4046</v>
       </c>
       <c r="O610" s="4" t="s">
-        <v>4687</v>
+        <v>4679</v>
       </c>
       <c r="P610" s="4" t="s">
-        <v>4688</v>
+        <v>4680</v>
       </c>
       <c r="Q610" s="4" t="b">
         <v>0</v>
@@ -70632,7 +70503,7 @@
     </row>
     <row r="611" spans="1:23" ht="30">
       <c r="A611" s="4" t="s">
-        <v>4634</v>
+        <v>4626</v>
       </c>
       <c r="B611" s="4">
         <v>13</v>
@@ -70665,13 +70536,13 @@
         <v>73</v>
       </c>
       <c r="N611" s="4" t="s">
-        <v>4689</v>
+        <v>4681</v>
       </c>
       <c r="O611" s="4" t="s">
-        <v>4690</v>
+        <v>4682</v>
       </c>
       <c r="P611" s="4" t="s">
-        <v>4691</v>
+        <v>4683</v>
       </c>
       <c r="Q611" s="4">
         <v>1</v>
@@ -73616,13 +73487,13 @@
         <v>267</v>
       </c>
       <c r="C97" s="4" t="s">
+        <v>4541</v>
+      </c>
+      <c r="D97" s="4" t="s">
         <v>4542</v>
       </c>
-      <c r="D97" s="4" t="s">
+      <c r="E97" s="4" t="s">
         <v>4543</v>
-      </c>
-      <c r="E97" s="4" t="s">
-        <v>4544</v>
       </c>
       <c r="F97" s="4">
         <v>1</v>
@@ -73634,7 +73505,7 @@
         <v>7</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>4545</v>
+        <v>4544</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="60">
@@ -73645,13 +73516,13 @@
         <v>267</v>
       </c>
       <c r="C98" s="4" t="s">
+        <v>4545</v>
+      </c>
+      <c r="D98" s="4" t="s">
         <v>4546</v>
       </c>
-      <c r="D98" s="4" t="s">
+      <c r="E98" s="4" t="s">
         <v>4547</v>
-      </c>
-      <c r="E98" s="4" t="s">
-        <v>4548</v>
       </c>
       <c r="F98" s="4">
         <v>2</v>
@@ -73663,7 +73534,7 @@
         <v>7</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>4549</v>
+        <v>4548</v>
       </c>
     </row>
     <row r="99" spans="1:9" ht="75">
@@ -73674,13 +73545,13 @@
         <v>267</v>
       </c>
       <c r="C99" s="4" t="s">
+        <v>4549</v>
+      </c>
+      <c r="D99" s="4" t="s">
         <v>4550</v>
       </c>
-      <c r="D99" s="4" t="s">
+      <c r="E99" s="4" t="s">
         <v>4551</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>4552</v>
       </c>
       <c r="F99" s="4">
         <v>3</v>
@@ -73692,7 +73563,7 @@
         <v>7</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>4553</v>
+        <v>4552</v>
       </c>
     </row>
     <row r="100" spans="1:9" ht="75">
@@ -73703,13 +73574,13 @@
         <v>267</v>
       </c>
       <c r="C100" s="4" t="s">
+        <v>4553</v>
+      </c>
+      <c r="D100" s="4" t="s">
         <v>4554</v>
       </c>
-      <c r="D100" s="4" t="s">
+      <c r="E100" s="4" t="s">
         <v>4555</v>
-      </c>
-      <c r="E100" s="4" t="s">
-        <v>4556</v>
       </c>
       <c r="F100" s="4">
         <v>4</v>
@@ -73721,7 +73592,7 @@
         <v>7</v>
       </c>
       <c r="I100" s="4" t="s">
-        <v>4557</v>
+        <v>4556</v>
       </c>
     </row>
     <row r="101" spans="1:9" ht="30">
@@ -73738,7 +73609,7 @@
         <v>715</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>4558</v>
+        <v>4557</v>
       </c>
       <c r="F101" s="4">
         <v>1</v>
@@ -73750,7 +73621,7 @@
         <v>7</v>
       </c>
       <c r="I101" s="4" t="s">
-        <v>4559</v>
+        <v>4558</v>
       </c>
     </row>
     <row r="102" spans="1:9" ht="30">
@@ -73761,13 +73632,13 @@
         <v>267</v>
       </c>
       <c r="C102" s="4" t="s">
+        <v>4559</v>
+      </c>
+      <c r="D102" s="4" t="s">
         <v>4560</v>
       </c>
-      <c r="D102" s="4" t="s">
+      <c r="E102" s="4" t="s">
         <v>4561</v>
-      </c>
-      <c r="E102" s="4" t="s">
-        <v>4562</v>
       </c>
       <c r="F102" s="4">
         <v>2</v>
@@ -73779,7 +73650,7 @@
         <v>7</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>4563</v>
+        <v>4562</v>
       </c>
     </row>
     <row r="103" spans="1:9" ht="60">
@@ -73793,10 +73664,10 @@
         <v>860</v>
       </c>
       <c r="D103" s="4" t="s">
+        <v>4563</v>
+      </c>
+      <c r="E103" s="4" t="s">
         <v>4564</v>
-      </c>
-      <c r="E103" s="4" t="s">
-        <v>4565</v>
       </c>
       <c r="F103" s="4">
         <v>3</v>
@@ -73808,7 +73679,7 @@
         <v>7</v>
       </c>
       <c r="I103" s="4" t="s">
-        <v>4566</v>
+        <v>4565</v>
       </c>
     </row>
     <row r="104" spans="1:9" ht="30">
@@ -73822,10 +73693,10 @@
         <v>871</v>
       </c>
       <c r="D104" s="4" t="s">
+        <v>4566</v>
+      </c>
+      <c r="E104" s="4" t="s">
         <v>4567</v>
-      </c>
-      <c r="E104" s="4" t="s">
-        <v>4568</v>
       </c>
       <c r="F104" s="4">
         <v>4</v>
@@ -73837,7 +73708,7 @@
         <v>7</v>
       </c>
       <c r="I104" s="4" t="s">
-        <v>4569</v>
+        <v>4568</v>
       </c>
     </row>
     <row r="105" spans="1:9" ht="75">
@@ -73848,13 +73719,13 @@
         <v>267</v>
       </c>
       <c r="C105" s="4" t="s">
+        <v>4569</v>
+      </c>
+      <c r="D105" s="4" t="s">
         <v>4570</v>
       </c>
-      <c r="D105" s="4" t="s">
+      <c r="E105" s="4" t="s">
         <v>4571</v>
-      </c>
-      <c r="E105" s="4" t="s">
-        <v>4572</v>
       </c>
       <c r="F105" s="4">
         <v>5</v>
@@ -73866,7 +73737,7 @@
         <v>7</v>
       </c>
       <c r="I105" s="4" t="s">
-        <v>4573</v>
+        <v>4572</v>
       </c>
     </row>
     <row r="106" spans="1:9" ht="75">
@@ -73877,25 +73748,25 @@
         <v>267</v>
       </c>
       <c r="C106" s="4" t="s">
+        <v>4573</v>
+      </c>
+      <c r="D106" s="4" t="s">
         <v>4574</v>
       </c>
-      <c r="D106" s="4" t="s">
+      <c r="E106" s="4" t="s">
         <v>4575</v>
       </c>
-      <c r="E106" s="4" t="s">
+      <c r="F106" s="4">
+        <v>6</v>
+      </c>
+      <c r="G106" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I106" s="4" t="s">
         <v>4576</v>
-      </c>
-      <c r="F106" s="4">
-        <v>6</v>
-      </c>
-      <c r="G106" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H106" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I106" s="4" t="s">
-        <v>4577</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Benefits server implementation complete
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67D07DE-ADBC-4683-8142-E13D3035F177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C013DA-A0B8-48DC-BEBD-227039E6FBD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="11" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">Relationships!$A$1:$K$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19511" uniqueCount="4930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19517" uniqueCount="4931">
   <si>
     <t>Domain</t>
   </si>
@@ -14834,6 +14835,9 @@
   </si>
   <si>
     <t>entity-status-member-benefit-inactive</t>
+  </si>
+  <si>
+    <t>BENEFIT_USAGE_RULE</t>
   </si>
 </sst>
 </file>
@@ -19607,7 +19611,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7B29B1-81FD-48F8-9727-C5470F35164D}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" style="4" bestFit="1" customWidth="1"/>
@@ -19979,6 +19983,34 @@
       </c>
       <c r="D26" s="4" t="s">
         <v>2218</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>4202</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>4930</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>2224</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>2410</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>2464</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2235</v>
       </c>
     </row>
   </sheetData>
@@ -25189,7 +25221,7 @@
         <v>4678</v>
       </c>
     </row>
-    <row r="101" spans="1:11">
+    <row r="101" spans="1:11" ht="30">
       <c r="A101" s="4" t="s">
         <v>4679</v>
       </c>
@@ -25224,7 +25256,7 @@
         <v>4602</v>
       </c>
     </row>
-    <row r="102" spans="1:11">
+    <row r="102" spans="1:11" ht="30">
       <c r="A102" s="4" t="s">
         <v>4680</v>
       </c>
@@ -25259,7 +25291,7 @@
         <v>4681</v>
       </c>
     </row>
-    <row r="103" spans="1:11">
+    <row r="103" spans="1:11" ht="30">
       <c r="A103" s="4" t="s">
         <v>4682</v>
       </c>
@@ -25294,7 +25326,7 @@
         <v>4605</v>
       </c>
     </row>
-    <row r="104" spans="1:11">
+    <row r="104" spans="1:11" ht="30">
       <c r="A104" s="4" t="s">
         <v>4683</v>
       </c>
@@ -25329,7 +25361,7 @@
         <v>4684</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
+    <row r="105" spans="1:11" ht="30">
       <c r="A105" s="4" t="s">
         <v>4685</v>
       </c>
@@ -25364,7 +25396,7 @@
         <v>4608</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" spans="1:11" ht="30">
       <c r="A106" s="4" t="s">
         <v>4686</v>
       </c>
@@ -25469,7 +25501,7 @@
         <v>4690</v>
       </c>
     </row>
-    <row r="109" spans="1:11">
+    <row r="109" spans="1:11" ht="30">
       <c r="A109" s="4" t="s">
         <v>4691</v>
       </c>
@@ -25504,7 +25536,7 @@
         <v>4614</v>
       </c>
     </row>
-    <row r="110" spans="1:11">
+    <row r="110" spans="1:11" ht="30">
       <c r="A110" s="4" t="s">
         <v>4692</v>
       </c>
@@ -25819,7 +25851,7 @@
         <v>4705</v>
       </c>
     </row>
-    <row r="119" spans="1:11">
+    <row r="119" spans="1:11" ht="30">
       <c r="A119" s="4" t="s">
         <v>4706</v>
       </c>
@@ -25854,7 +25886,7 @@
         <v>4629</v>
       </c>
     </row>
-    <row r="120" spans="1:11">
+    <row r="120" spans="1:11" ht="30">
       <c r="A120" s="4" t="s">
         <v>4707</v>
       </c>
@@ -25889,7 +25921,7 @@
         <v>4708</v>
       </c>
     </row>
-    <row r="121" spans="1:11">
+    <row r="121" spans="1:11" ht="30">
       <c r="A121" s="4" t="s">
         <v>4709</v>
       </c>
@@ -25924,7 +25956,7 @@
         <v>4632</v>
       </c>
     </row>
-    <row r="122" spans="1:11">
+    <row r="122" spans="1:11" ht="30">
       <c r="A122" s="4" t="s">
         <v>4710</v>
       </c>
@@ -25959,7 +25991,7 @@
         <v>4711</v>
       </c>
     </row>
-    <row r="123" spans="1:11">
+    <row r="123" spans="1:11" ht="30">
       <c r="A123" s="4" t="s">
         <v>4712</v>
       </c>
@@ -25994,7 +26026,7 @@
         <v>4635</v>
       </c>
     </row>
-    <row r="124" spans="1:11">
+    <row r="124" spans="1:11" ht="30">
       <c r="A124" s="4" t="s">
         <v>4713</v>
       </c>
@@ -26029,7 +26061,7 @@
         <v>4714</v>
       </c>
     </row>
-    <row r="125" spans="1:11">
+    <row r="125" spans="1:11" ht="30">
       <c r="A125" s="4" t="s">
         <v>4715</v>
       </c>
@@ -26064,7 +26096,7 @@
         <v>4717</v>
       </c>
     </row>
-    <row r="126" spans="1:11">
+    <row r="126" spans="1:11" ht="30">
       <c r="A126" s="4" t="s">
         <v>4718</v>
       </c>
@@ -26099,7 +26131,7 @@
         <v>4720</v>
       </c>
     </row>
-    <row r="127" spans="1:11">
+    <row r="127" spans="1:11" ht="30">
       <c r="A127" s="4" t="s">
         <v>4721</v>
       </c>
@@ -26134,7 +26166,7 @@
         <v>4723</v>
       </c>
     </row>
-    <row r="128" spans="1:11">
+    <row r="128" spans="1:11" ht="30">
       <c r="A128" s="4" t="s">
         <v>4724</v>
       </c>
@@ -26239,7 +26271,7 @@
         <v>4729</v>
       </c>
     </row>
-    <row r="131" spans="1:11">
+    <row r="131" spans="1:11" ht="30">
       <c r="A131" s="4" t="s">
         <v>4730</v>
       </c>
@@ -26274,7 +26306,7 @@
         <v>4641</v>
       </c>
     </row>
-    <row r="132" spans="1:11">
+    <row r="132" spans="1:11" ht="30">
       <c r="A132" s="4" t="s">
         <v>4731</v>
       </c>
@@ -26309,7 +26341,7 @@
         <v>4732</v>
       </c>
     </row>
-    <row r="133" spans="1:11">
+    <row r="133" spans="1:11" ht="30">
       <c r="A133" s="4" t="s">
         <v>4733</v>
       </c>
@@ -26344,7 +26376,7 @@
         <v>4644</v>
       </c>
     </row>
-    <row r="134" spans="1:11">
+    <row r="134" spans="1:11" ht="30">
       <c r="A134" s="4" t="s">
         <v>4734</v>
       </c>
@@ -26449,7 +26481,7 @@
         <v>4738</v>
       </c>
     </row>
-    <row r="137" spans="1:11">
+    <row r="137" spans="1:11" ht="30">
       <c r="A137" s="4" t="s">
         <v>4739</v>
       </c>
@@ -26484,7 +26516,7 @@
         <v>4650</v>
       </c>
     </row>
-    <row r="138" spans="1:11">
+    <row r="138" spans="1:11" ht="30">
       <c r="A138" s="4" t="s">
         <v>4740</v>
       </c>
@@ -26589,7 +26621,7 @@
         <v>4744</v>
       </c>
     </row>
-    <row r="141" spans="1:11">
+    <row r="141" spans="1:11" ht="30">
       <c r="A141" s="4" t="s">
         <v>4745</v>
       </c>
@@ -26624,7 +26656,7 @@
         <v>4656</v>
       </c>
     </row>
-    <row r="142" spans="1:11">
+    <row r="142" spans="1:11" ht="30">
       <c r="A142" s="4" t="s">
         <v>4746</v>
       </c>
@@ -26764,7 +26796,7 @@
         <v>4662</v>
       </c>
     </row>
-    <row r="146" spans="1:11">
+    <row r="146" spans="1:11" ht="30">
       <c r="A146" s="4" t="s">
         <v>4752</v>
       </c>
@@ -26799,7 +26831,7 @@
         <v>4753</v>
       </c>
     </row>
-    <row r="147" spans="1:11">
+    <row r="147" spans="1:11" ht="30">
       <c r="A147" s="4" t="s">
         <v>4754</v>
       </c>
@@ -26834,7 +26866,7 @@
         <v>4665</v>
       </c>
     </row>
-    <row r="148" spans="1:11">
+    <row r="148" spans="1:11" ht="30">
       <c r="A148" s="4" t="s">
         <v>4755</v>
       </c>
@@ -26869,7 +26901,7 @@
         <v>4756</v>
       </c>
     </row>
-    <row r="149" spans="1:11">
+    <row r="149" spans="1:11" ht="30">
       <c r="A149" s="4" t="s">
         <v>4757</v>
       </c>
@@ -26904,7 +26936,7 @@
         <v>4759</v>
       </c>
     </row>
-    <row r="150" spans="1:11">
+    <row r="150" spans="1:11" ht="30">
       <c r="A150" s="4" t="s">
         <v>4760</v>
       </c>
@@ -26939,7 +26971,7 @@
         <v>4668</v>
       </c>
     </row>
-    <row r="151" spans="1:11">
+    <row r="151" spans="1:11" ht="30">
       <c r="A151" s="4" t="s">
         <v>4761</v>
       </c>
@@ -27044,7 +27076,7 @@
         <v>4766</v>
       </c>
     </row>
-    <row r="154" spans="1:11">
+    <row r="154" spans="1:11" ht="30">
       <c r="A154" s="4" t="s">
         <v>4767</v>
       </c>
@@ -27429,7 +27461,7 @@
         <v>4797</v>
       </c>
     </row>
-    <row r="165" spans="1:11">
+    <row r="165" spans="1:11" ht="30">
       <c r="A165" s="4" t="s">
         <v>4798</v>
       </c>
@@ -27464,7 +27496,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="166" spans="1:11">
+    <row r="166" spans="1:11" ht="30">
       <c r="A166" s="4" t="s">
         <v>4801</v>
       </c>
@@ -27569,7 +27601,7 @@
         <v>4809</v>
       </c>
     </row>
-    <row r="169" spans="1:11">
+    <row r="169" spans="1:11" ht="30">
       <c r="A169" s="4" t="s">
         <v>4810</v>
       </c>
@@ -27639,7 +27671,7 @@
         <v>4815</v>
       </c>
     </row>
-    <row r="171" spans="1:11">
+    <row r="171" spans="1:11" ht="30">
       <c r="A171" s="4" t="s">
         <v>4816</v>
       </c>
@@ -27674,7 +27706,7 @@
         <v>4818</v>
       </c>
     </row>
-    <row r="172" spans="1:11">
+    <row r="172" spans="1:11" ht="30">
       <c r="A172" s="4" t="s">
         <v>4819</v>
       </c>
@@ -27709,7 +27741,7 @@
         <v>4820</v>
       </c>
     </row>
-    <row r="173" spans="1:11">
+    <row r="173" spans="1:11" ht="30">
       <c r="A173" s="4" t="s">
         <v>4821</v>
       </c>
@@ -27744,7 +27776,7 @@
         <v>4823</v>
       </c>
     </row>
-    <row r="174" spans="1:11">
+    <row r="174" spans="1:11" ht="30">
       <c r="A174" s="4" t="s">
         <v>4824</v>
       </c>
@@ -32100,7 +32132,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="30">
+    <row r="2" spans="1:23" ht="30" hidden="1">
       <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
@@ -32304,7 +32336,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="45">
+    <row r="5" spans="1:23" ht="45" hidden="1">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -32512,7 +32544,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" hidden="1">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -32580,7 +32612,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" hidden="1">
       <c r="A9" s="10" t="s">
         <v>5</v>
       </c>
@@ -32920,7 +32952,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23">
+    <row r="14" spans="1:23" hidden="1">
       <c r="A14" s="10" t="s">
         <v>5</v>
       </c>
@@ -33056,7 +33088,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:23">
+    <row r="16" spans="1:23" hidden="1">
       <c r="A16" s="10" t="s">
         <v>5</v>
       </c>
@@ -33260,7 +33292,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="30">
+    <row r="19" spans="1:23" ht="30" hidden="1">
       <c r="A19" s="3" t="s">
         <v>8</v>
       </c>
@@ -33802,7 +33834,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="30">
+    <row r="27" spans="1:23" ht="30" hidden="1">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -33873,7 +33905,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="30">
+    <row r="28" spans="1:23" ht="30" hidden="1">
       <c r="A28" s="3" t="s">
         <v>8</v>
       </c>
@@ -34011,7 +34043,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:23" hidden="1">
       <c r="A30" s="3" t="s">
         <v>8</v>
       </c>
@@ -34149,7 +34181,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:23" hidden="1">
       <c r="A32" s="3" t="s">
         <v>8</v>
       </c>
@@ -34354,7 +34386,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="30">
+    <row r="35" spans="1:23" ht="30" hidden="1">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -34425,7 +34457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="30">
+    <row r="36" spans="1:23" ht="30" hidden="1">
       <c r="A36" s="3" t="s">
         <v>37</v>
       </c>
@@ -34496,7 +34528,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:23">
+    <row r="37" spans="1:23" hidden="1">
       <c r="A37" s="3" t="s">
         <v>37</v>
       </c>
@@ -34567,7 +34599,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="45">
+    <row r="38" spans="1:23" ht="45" hidden="1">
       <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
@@ -34638,7 +34670,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="30">
+    <row r="39" spans="1:23" ht="30" hidden="1">
       <c r="A39" s="3" t="s">
         <v>37</v>
       </c>
@@ -34851,7 +34883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:23">
+    <row r="42" spans="1:23" hidden="1">
       <c r="A42" s="3" t="s">
         <v>37</v>
       </c>
@@ -34993,7 +35025,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:23">
+    <row r="44" spans="1:23" hidden="1">
       <c r="A44" s="3" t="s">
         <v>37</v>
       </c>
@@ -35206,7 +35238,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="30">
+    <row r="47" spans="1:23" ht="30" hidden="1">
       <c r="A47" s="3" t="s">
         <v>315</v>
       </c>
@@ -35394,7 +35426,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="30">
+    <row r="51" spans="1:23" ht="30" hidden="1">
       <c r="A51" s="3" t="s">
         <v>315</v>
       </c>
@@ -35441,7 +35473,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="30">
+    <row r="52" spans="1:23" ht="30" hidden="1">
       <c r="A52" s="4" t="s">
         <v>339</v>
       </c>
@@ -35509,7 +35541,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="30">
+    <row r="53" spans="1:23" ht="30" hidden="1">
       <c r="A53" s="4" t="s">
         <v>339</v>
       </c>
@@ -35577,7 +35609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="30">
+    <row r="54" spans="1:23" ht="30" hidden="1">
       <c r="A54" s="4" t="s">
         <v>339</v>
       </c>
@@ -35645,7 +35677,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="30">
+    <row r="55" spans="1:23" ht="30" hidden="1">
       <c r="A55" s="4" t="s">
         <v>339</v>
       </c>
@@ -35781,7 +35813,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="30">
+    <row r="57" spans="1:23" ht="30" hidden="1">
       <c r="A57" s="4" t="s">
         <v>339</v>
       </c>
@@ -35917,7 +35949,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="30">
+    <row r="59" spans="1:23" ht="30" hidden="1">
       <c r="A59" s="4" t="s">
         <v>339</v>
       </c>
@@ -36121,7 +36153,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="30">
+    <row r="62" spans="1:23" ht="30" hidden="1">
       <c r="A62" s="4" t="s">
         <v>368</v>
       </c>
@@ -36405,7 +36437,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="30">
+    <row r="66" spans="1:23" ht="30" hidden="1">
       <c r="A66" s="4" t="s">
         <v>368</v>
       </c>
@@ -36476,7 +36508,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="30">
+    <row r="67" spans="1:23" ht="30" hidden="1">
       <c r="A67" s="4" t="s">
         <v>375</v>
       </c>
@@ -36547,7 +36579,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="30">
+    <row r="68" spans="1:23" ht="30" hidden="1">
       <c r="A68" s="4" t="s">
         <v>375</v>
       </c>
@@ -36618,7 +36650,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="30">
+    <row r="69" spans="1:23" ht="30" hidden="1">
       <c r="A69" s="4" t="s">
         <v>375</v>
       </c>
@@ -36689,7 +36721,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="30">
+    <row r="70" spans="1:23" ht="30" hidden="1">
       <c r="A70" s="4" t="s">
         <v>10</v>
       </c>
@@ -36760,7 +36792,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="30">
+    <row r="71" spans="1:23" ht="30" hidden="1">
       <c r="A71" s="4" t="s">
         <v>10</v>
       </c>
@@ -37044,7 +37076,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="30">
+    <row r="75" spans="1:23" ht="30" hidden="1">
       <c r="A75" s="4" t="s">
         <v>10</v>
       </c>
@@ -37115,7 +37147,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="30">
+    <row r="76" spans="1:23" ht="30" hidden="1">
       <c r="A76" s="4" t="s">
         <v>10</v>
       </c>
@@ -37257,7 +37289,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="30">
+    <row r="78" spans="1:23" ht="30" hidden="1">
       <c r="A78" s="4" t="s">
         <v>10</v>
       </c>
@@ -37683,7 +37715,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="30">
+    <row r="84" spans="1:23" ht="30" hidden="1">
       <c r="A84" s="4" t="s">
         <v>10</v>
       </c>
@@ -37825,7 +37857,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="30">
+    <row r="86" spans="1:23" ht="30" hidden="1">
       <c r="A86" s="4" t="s">
         <v>10</v>
       </c>
@@ -38038,7 +38070,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="30">
+    <row r="89" spans="1:23" ht="30" hidden="1">
       <c r="A89" s="4" t="s">
         <v>488</v>
       </c>
@@ -38322,7 +38354,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:23">
+    <row r="93" spans="1:23" hidden="1">
       <c r="A93" s="4" t="s">
         <v>488</v>
       </c>
@@ -38393,7 +38425,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:23">
+    <row r="94" spans="1:23" hidden="1">
       <c r="A94" s="4" t="s">
         <v>488</v>
       </c>
@@ -38535,7 +38567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30">
+    <row r="96" spans="1:23" ht="30" hidden="1">
       <c r="A96" s="4" t="s">
         <v>488</v>
       </c>
@@ -38606,7 +38638,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="30">
+    <row r="97" spans="1:23" ht="30" hidden="1">
       <c r="A97" s="4" t="s">
         <v>488</v>
       </c>
@@ -39032,7 +39064,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="30">
+    <row r="103" spans="1:23" ht="30" hidden="1">
       <c r="A103" s="4" t="s">
         <v>488</v>
       </c>
@@ -39174,7 +39206,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="30">
+    <row r="105" spans="1:23" ht="30" hidden="1">
       <c r="A105" s="4" t="s">
         <v>488</v>
       </c>
@@ -39387,7 +39419,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="30">
+    <row r="108" spans="1:23" ht="30" hidden="1">
       <c r="A108" s="4" t="s">
         <v>546</v>
       </c>
@@ -39458,7 +39490,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="30">
+    <row r="109" spans="1:23" ht="30" hidden="1">
       <c r="A109" s="4" t="s">
         <v>546</v>
       </c>
@@ -39955,7 +39987,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="30">
+    <row r="116" spans="1:23" ht="30" hidden="1">
       <c r="A116" s="4" t="s">
         <v>546</v>
       </c>
@@ -40026,7 +40058,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:23">
+    <row r="117" spans="1:23" hidden="1">
       <c r="A117" s="4" t="s">
         <v>546</v>
       </c>
@@ -40310,7 +40342,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:23">
+    <row r="121" spans="1:23" hidden="1">
       <c r="A121" s="4" t="s">
         <v>546</v>
       </c>
@@ -40452,7 +40484,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:23">
+    <row r="123" spans="1:23" hidden="1">
       <c r="A123" s="4" t="s">
         <v>546</v>
       </c>
@@ -40665,7 +40697,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="30">
+    <row r="126" spans="1:23" ht="30" hidden="1">
       <c r="A126" s="4" t="s">
         <v>618</v>
       </c>
@@ -40807,7 +40839,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:23">
+    <row r="128" spans="1:23" hidden="1">
       <c r="A128" s="4" t="s">
         <v>618</v>
       </c>
@@ -40878,7 +40910,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="30">
+    <row r="129" spans="1:23" ht="30" hidden="1">
       <c r="A129" s="4" t="s">
         <v>618</v>
       </c>
@@ -41162,7 +41194,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="1:23">
+    <row r="133" spans="1:23" hidden="1">
       <c r="A133" s="4" t="s">
         <v>618</v>
       </c>
@@ -41375,7 +41407,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="136" spans="1:23">
+    <row r="136" spans="1:23" hidden="1">
       <c r="A136" s="4" t="s">
         <v>618</v>
       </c>
@@ -41517,7 +41549,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:23">
+    <row r="138" spans="1:23" hidden="1">
       <c r="A138" s="4" t="s">
         <v>618</v>
       </c>
@@ -41730,7 +41762,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="30">
+    <row r="141" spans="1:23" ht="30" hidden="1">
       <c r="A141" s="4" t="s">
         <v>671</v>
       </c>
@@ -41872,7 +41904,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="30">
+    <row r="143" spans="1:23" ht="30" hidden="1">
       <c r="A143" s="4" t="s">
         <v>671</v>
       </c>
@@ -41943,7 +41975,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="30">
+    <row r="144" spans="1:23" ht="30" hidden="1">
       <c r="A144" s="4" t="s">
         <v>671</v>
       </c>
@@ -42014,7 +42046,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="30">
+    <row r="145" spans="1:23" ht="30" hidden="1">
       <c r="A145" s="4" t="s">
         <v>671</v>
       </c>
@@ -42085,7 +42117,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="30">
+    <row r="146" spans="1:23" ht="30" hidden="1">
       <c r="A146" s="4" t="s">
         <v>671</v>
       </c>
@@ -42298,7 +42330,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="30">
+    <row r="149" spans="1:23" ht="30" hidden="1">
       <c r="A149" s="4" t="s">
         <v>671</v>
       </c>
@@ -42511,7 +42543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="30">
+    <row r="152" spans="1:23" ht="30" hidden="1">
       <c r="A152" s="4" t="s">
         <v>671</v>
       </c>
@@ -42653,7 +42685,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="30">
+    <row r="154" spans="1:23" ht="30" hidden="1">
       <c r="A154" s="4" t="s">
         <v>671</v>
       </c>
@@ -42795,7 +42827,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="30">
+    <row r="156" spans="1:23" ht="30" hidden="1">
       <c r="A156" s="4" t="s">
         <v>34</v>
       </c>
@@ -42866,7 +42898,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="30">
+    <row r="157" spans="1:23" ht="30" hidden="1">
       <c r="A157" s="4" t="s">
         <v>34</v>
       </c>
@@ -43079,7 +43111,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:23">
+    <row r="160" spans="1:23" hidden="1">
       <c r="A160" s="4" t="s">
         <v>34</v>
       </c>
@@ -43789,7 +43821,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="30">
+    <row r="170" spans="1:23" ht="30" hidden="1">
       <c r="A170" s="4" t="s">
         <v>34</v>
       </c>
@@ -44073,7 +44105,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="1:23">
+    <row r="174" spans="1:23" hidden="1">
       <c r="A174" s="4" t="s">
         <v>34</v>
       </c>
@@ -44215,7 +44247,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="30">
+    <row r="176" spans="1:23" ht="30" hidden="1">
       <c r="A176" s="4" t="s">
         <v>34</v>
       </c>
@@ -44428,7 +44460,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="30">
+    <row r="179" spans="1:23" ht="30" hidden="1">
       <c r="A179" s="4" t="s">
         <v>35</v>
       </c>
@@ -44499,7 +44531,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="30">
+    <row r="180" spans="1:23" ht="30" hidden="1">
       <c r="A180" s="4" t="s">
         <v>35</v>
       </c>
@@ -44641,7 +44673,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="30">
+    <row r="182" spans="1:23" ht="30" hidden="1">
       <c r="A182" s="3" t="s">
         <v>35</v>
       </c>
@@ -44712,7 +44744,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="30">
+    <row r="183" spans="1:23" ht="30" hidden="1">
       <c r="A183" s="3" t="s">
         <v>35</v>
       </c>
@@ -44854,7 +44886,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="30">
+    <row r="185" spans="1:23" ht="30" hidden="1">
       <c r="A185" s="4" t="s">
         <v>35</v>
       </c>
@@ -45067,7 +45099,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="30">
+    <row r="188" spans="1:23" ht="30" hidden="1">
       <c r="A188" s="4" t="s">
         <v>35</v>
       </c>
@@ -45209,7 +45241,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="30">
+    <row r="190" spans="1:23" ht="30" hidden="1">
       <c r="A190" s="4" t="s">
         <v>35</v>
       </c>
@@ -45351,7 +45383,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="30">
+    <row r="192" spans="1:23" ht="30" hidden="1">
       <c r="A192" s="4" t="s">
         <v>35</v>
       </c>
@@ -45564,7 +45596,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="195" spans="1:23" ht="30">
+    <row r="195" spans="1:23" ht="30" hidden="1">
       <c r="A195" s="3" t="s">
         <v>94</v>
       </c>
@@ -45978,7 +46010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="201" spans="1:23">
+    <row r="201" spans="1:23" hidden="1">
       <c r="A201" s="3" t="s">
         <v>42</v>
       </c>
@@ -46392,7 +46424,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="207" spans="1:23">
+    <row r="207" spans="1:23" hidden="1">
       <c r="A207" s="3" t="s">
         <v>129</v>
       </c>
@@ -46875,7 +46907,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="214" spans="1:23">
+    <row r="214" spans="1:23" hidden="1">
       <c r="A214" s="3" t="s">
         <v>126</v>
       </c>
@@ -47427,7 +47459,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="222" spans="1:23" ht="30">
+    <row r="222" spans="1:23" ht="30" hidden="1">
       <c r="A222" s="3" t="s">
         <v>311</v>
       </c>
@@ -47841,7 +47873,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="228" spans="1:23" ht="30">
+    <row r="228" spans="1:23" ht="30" hidden="1">
       <c r="A228" s="3" t="s">
         <v>443</v>
       </c>
@@ -48255,7 +48287,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="234" spans="1:23" ht="30">
+    <row r="234" spans="1:23" ht="30" hidden="1">
       <c r="A234" s="3" t="s">
         <v>449</v>
       </c>
@@ -48669,7 +48701,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="240" spans="1:23" ht="30">
+    <row r="240" spans="1:23" ht="30" hidden="1">
       <c r="A240" s="3" t="s">
         <v>510</v>
       </c>
@@ -49083,7 +49115,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="246" spans="1:23" ht="30">
+    <row r="246" spans="1:23" ht="30" hidden="1">
       <c r="A246" s="3" t="s">
         <v>516</v>
       </c>
@@ -49497,7 +49529,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="252" spans="1:23" ht="30">
+    <row r="252" spans="1:23" ht="30" hidden="1">
       <c r="A252" s="3" t="s">
         <v>754</v>
       </c>
@@ -49911,7 +49943,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="258" spans="1:23" ht="30">
+    <row r="258" spans="1:23" ht="30" hidden="1">
       <c r="A258" s="3" t="s">
         <v>1502</v>
       </c>
@@ -49980,7 +50012,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="259" spans="1:23" ht="30">
+    <row r="259" spans="1:23" ht="30" hidden="1">
       <c r="A259" s="3" t="s">
         <v>1502</v>
       </c>
@@ -50877,7 +50909,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="272" spans="1:23">
+    <row r="272" spans="1:23" hidden="1">
       <c r="A272" s="3" t="s">
         <v>1502</v>
       </c>
@@ -51013,7 +51045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="274" spans="1:23">
+    <row r="274" spans="1:23" hidden="1">
       <c r="A274" s="3" t="s">
         <v>1502</v>
       </c>
@@ -51220,7 +51252,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="277" spans="1:23" ht="30">
+    <row r="277" spans="1:23" ht="30" hidden="1">
       <c r="A277" s="3" t="s">
         <v>1503</v>
       </c>
@@ -51289,7 +51321,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="278" spans="1:23" ht="30">
+    <row r="278" spans="1:23" ht="30" hidden="1">
       <c r="A278" s="3" t="s">
         <v>1503</v>
       </c>
@@ -51429,7 +51461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="280" spans="1:23">
+    <row r="280" spans="1:23" hidden="1">
       <c r="A280" s="3" t="s">
         <v>1503</v>
       </c>
@@ -51981,7 +52013,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="288" spans="1:23" ht="30">
+    <row r="288" spans="1:23" ht="30" hidden="1">
       <c r="A288" s="3" t="s">
         <v>1503</v>
       </c>
@@ -52231,7 +52263,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="292" spans="1:23">
+    <row r="292" spans="1:23" hidden="1">
       <c r="A292" s="3" t="s">
         <v>1503</v>
       </c>
@@ -52363,7 +52395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="294" spans="1:23">
+    <row r="294" spans="1:23" hidden="1">
       <c r="A294" s="3" t="s">
         <v>1503</v>
       </c>
@@ -52568,7 +52600,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="297" spans="1:23" ht="30">
+    <row r="297" spans="1:23" ht="30" hidden="1">
       <c r="A297" s="3" t="s">
         <v>1563</v>
       </c>
@@ -52637,7 +52669,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="298" spans="1:23" ht="30">
+    <row r="298" spans="1:23" ht="30" hidden="1">
       <c r="A298" s="3" t="s">
         <v>1563</v>
       </c>
@@ -53122,7 +53154,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="305" spans="1:23" ht="30">
+    <row r="305" spans="1:23" ht="30" hidden="1">
       <c r="A305" s="3" t="s">
         <v>1563</v>
       </c>
@@ -53258,7 +53290,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="307" spans="1:23" ht="30">
+    <row r="307" spans="1:23" ht="30" hidden="1">
       <c r="A307" s="3" t="s">
         <v>1563</v>
       </c>
@@ -53390,7 +53422,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="309" spans="1:23" ht="30">
+    <row r="309" spans="1:23" ht="30" hidden="1">
       <c r="A309" s="3" t="s">
         <v>1563</v>
       </c>
@@ -53595,7 +53627,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="312" spans="1:23" ht="30">
+    <row r="312" spans="1:23" ht="30" hidden="1">
       <c r="A312" s="3" t="s">
         <v>1620</v>
       </c>
@@ -53664,7 +53696,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="313" spans="1:23" ht="30">
+    <row r="313" spans="1:23" ht="30" hidden="1">
       <c r="A313" s="3" t="s">
         <v>1620</v>
       </c>
@@ -53869,7 +53901,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="316" spans="1:23">
+    <row r="316" spans="1:23" hidden="1">
       <c r="A316" s="3" t="s">
         <v>1620</v>
       </c>
@@ -54005,7 +54037,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="318" spans="1:23">
+    <row r="318" spans="1:23" hidden="1">
       <c r="A318" s="3" t="s">
         <v>1620</v>
       </c>
@@ -54344,7 +54376,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="323" spans="1:23" ht="30">
+    <row r="323" spans="1:23" ht="30" hidden="1">
       <c r="A323" s="3" t="s">
         <v>1674</v>
       </c>
@@ -54413,7 +54445,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="324" spans="1:23" ht="30">
+    <row r="324" spans="1:23" ht="30" hidden="1">
       <c r="A324" s="3" t="s">
         <v>1674</v>
       </c>
@@ -54551,7 +54583,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="326" spans="1:23" ht="30">
+    <row r="326" spans="1:23" ht="30" hidden="1">
       <c r="A326" s="3" t="s">
         <v>1674</v>
       </c>
@@ -54689,7 +54721,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="328" spans="1:23" ht="30">
+    <row r="328" spans="1:23" ht="30" hidden="1">
       <c r="A328" s="3" t="s">
         <v>1674</v>
       </c>
@@ -54827,7 +54859,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="330" spans="1:23" ht="30">
+    <row r="330" spans="1:23" ht="30" hidden="1">
       <c r="A330" s="3" t="s">
         <v>1674</v>
       </c>
@@ -54961,7 +54993,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="332" spans="1:23" ht="30">
+    <row r="332" spans="1:23" ht="30" hidden="1">
       <c r="A332" s="3" t="s">
         <v>1674</v>
       </c>
@@ -55168,7 +55200,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="335" spans="1:23" ht="30">
+    <row r="335" spans="1:23" ht="30" hidden="1">
       <c r="A335" s="3" t="s">
         <v>1689</v>
       </c>
@@ -55513,7 +55545,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="340" spans="1:23" ht="30">
+    <row r="340" spans="1:23" ht="30" hidden="1">
       <c r="A340" s="3" t="s">
         <v>1689</v>
       </c>
@@ -55854,7 +55886,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="345" spans="1:23" ht="30">
+    <row r="345" spans="1:23" ht="30" hidden="1">
       <c r="A345" s="3" t="s">
         <v>1790</v>
       </c>
@@ -55923,7 +55955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="346" spans="1:23" ht="30">
+    <row r="346" spans="1:23" ht="30" hidden="1">
       <c r="A346" s="3" t="s">
         <v>1790</v>
       </c>
@@ -55992,7 +56024,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="347" spans="1:23" ht="30">
+    <row r="347" spans="1:23" ht="30" hidden="1">
       <c r="A347" s="3" t="s">
         <v>1790</v>
       </c>
@@ -56333,7 +56365,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="352" spans="1:23" ht="30">
+    <row r="352" spans="1:23" ht="30" hidden="1">
       <c r="A352" s="3" t="s">
         <v>1790</v>
       </c>
@@ -56471,7 +56503,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="354" spans="1:23" ht="30">
+    <row r="354" spans="1:23" ht="30" hidden="1">
       <c r="A354" s="3" t="s">
         <v>1790</v>
       </c>
@@ -56605,7 +56637,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="356" spans="1:23" ht="30">
+    <row r="356" spans="1:23" ht="30" hidden="1">
       <c r="A356" s="3" t="s">
         <v>1790</v>
       </c>
@@ -56812,7 +56844,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="359" spans="1:23">
+    <row r="359" spans="1:23" hidden="1">
       <c r="A359" s="3" t="s">
         <v>1898</v>
       </c>
@@ -56881,7 +56913,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="360" spans="1:23">
+    <row r="360" spans="1:23" hidden="1">
       <c r="A360" s="3" t="s">
         <v>1898</v>
       </c>
@@ -57019,7 +57051,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="362" spans="1:23" ht="30">
+    <row r="362" spans="1:23" ht="30" hidden="1">
       <c r="A362" s="3" t="s">
         <v>1898</v>
       </c>
@@ -57368,7 +57400,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="367" spans="1:23" ht="30">
+    <row r="367" spans="1:23" ht="30" hidden="1">
       <c r="A367" s="3" t="s">
         <v>1898</v>
       </c>
@@ -57581,7 +57613,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="370" spans="1:23">
+    <row r="370" spans="1:23" hidden="1">
       <c r="A370" s="3" t="s">
         <v>1898</v>
       </c>
@@ -57721,7 +57753,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="372" spans="1:23" ht="30">
+    <row r="372" spans="1:23" ht="30" hidden="1">
       <c r="A372" s="3" t="s">
         <v>1898</v>
       </c>
@@ -57932,7 +57964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="375" spans="1:23" ht="30">
+    <row r="375" spans="1:23" ht="30" hidden="1">
       <c r="A375" s="3" t="s">
         <v>1906</v>
       </c>
@@ -58208,7 +58240,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="379" spans="1:23" ht="30">
+    <row r="379" spans="1:23" ht="30" hidden="1">
       <c r="A379" s="3" t="s">
         <v>1906</v>
       </c>
@@ -58279,7 +58311,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="380" spans="1:23" ht="30">
+    <row r="380" spans="1:23" ht="30" hidden="1">
       <c r="A380" s="4" t="s">
         <v>2001</v>
       </c>
@@ -58350,7 +58382,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="381" spans="1:23" ht="30">
+    <row r="381" spans="1:23" ht="30" hidden="1">
       <c r="A381" s="4" t="s">
         <v>2001</v>
       </c>
@@ -58421,7 +58453,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="382" spans="1:23" ht="30">
+    <row r="382" spans="1:23" ht="30" hidden="1">
       <c r="A382" s="4" t="s">
         <v>2001</v>
       </c>
@@ -58492,7 +58524,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="383" spans="1:23" ht="45">
+    <row r="383" spans="1:23" ht="45" hidden="1">
       <c r="A383" s="4" t="s">
         <v>2001</v>
       </c>
@@ -58634,7 +58666,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="385" spans="1:23" ht="30">
+    <row r="385" spans="1:23" ht="30" hidden="1">
       <c r="A385" s="4" t="s">
         <v>2001</v>
       </c>
@@ -58776,7 +58808,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="387" spans="1:23" ht="30">
+    <row r="387" spans="1:23" ht="30" hidden="1">
       <c r="A387" s="4" t="s">
         <v>2001</v>
       </c>
@@ -58989,7 +59021,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="390" spans="1:23" ht="30">
+    <row r="390" spans="1:23" ht="30" hidden="1">
       <c r="A390" s="4" t="s">
         <v>2045</v>
       </c>
@@ -59060,7 +59092,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="391" spans="1:23" ht="30">
+    <row r="391" spans="1:23" ht="30" hidden="1">
       <c r="A391" s="4" t="s">
         <v>2045</v>
       </c>
@@ -59131,7 +59163,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="392" spans="1:23" ht="30">
+    <row r="392" spans="1:23" ht="30" hidden="1">
       <c r="A392" s="4" t="s">
         <v>2045</v>
       </c>
@@ -59202,7 +59234,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="393" spans="1:23" ht="30">
+    <row r="393" spans="1:23" ht="30" hidden="1">
       <c r="A393" s="4" t="s">
         <v>2045</v>
       </c>
@@ -59486,7 +59518,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="397" spans="1:23" ht="30">
+    <row r="397" spans="1:23" ht="30" hidden="1">
       <c r="A397" s="4" t="s">
         <v>2045</v>
       </c>
@@ -59628,7 +59660,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="399" spans="1:23" ht="30">
+    <row r="399" spans="1:23" ht="30" hidden="1">
       <c r="A399" s="4" t="s">
         <v>2045</v>
       </c>
@@ -59841,7 +59873,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="402" spans="1:23">
+    <row r="402" spans="1:23" hidden="1">
       <c r="A402" s="4" t="s">
         <v>2093</v>
       </c>
@@ -59912,7 +59944,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="403" spans="1:23" ht="30">
+    <row r="403" spans="1:23" ht="30" hidden="1">
       <c r="A403" s="4" t="s">
         <v>2093</v>
       </c>
@@ -60190,7 +60222,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="407" spans="1:23" ht="45">
+    <row r="407" spans="1:23" ht="45" hidden="1">
       <c r="A407" s="4" t="s">
         <v>2093</v>
       </c>
@@ -60261,7 +60293,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="408" spans="1:23" ht="30">
+    <row r="408" spans="1:23" ht="30" hidden="1">
       <c r="A408" s="4" t="s">
         <v>2093</v>
       </c>
@@ -60962,7 +60994,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="418" spans="1:23" ht="30">
+    <row r="418" spans="1:23" ht="30" hidden="1">
       <c r="A418" s="4" t="s">
         <v>2093</v>
       </c>
@@ -61104,7 +61136,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="420" spans="1:23" ht="30">
+    <row r="420" spans="1:23" ht="30" hidden="1">
       <c r="A420" s="4" t="s">
         <v>2093</v>
       </c>
@@ -61246,7 +61278,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="422" spans="1:23" ht="30">
+    <row r="422" spans="1:23" ht="30" hidden="1">
       <c r="A422" s="4" t="s">
         <v>2093</v>
       </c>
@@ -61459,7 +61491,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="425" spans="1:23" ht="45">
+    <row r="425" spans="1:23" ht="45" hidden="1">
       <c r="A425" s="3" t="s">
         <v>2333</v>
       </c>
@@ -61530,7 +61562,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="426" spans="1:23" ht="30">
+    <row r="426" spans="1:23" ht="30" hidden="1">
       <c r="A426" s="3" t="s">
         <v>2333</v>
       </c>
@@ -61601,7 +61633,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="427" spans="1:23" ht="45">
+    <row r="427" spans="1:23" ht="45" hidden="1">
       <c r="A427" s="3" t="s">
         <v>2333</v>
       </c>
@@ -61814,7 +61846,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="430" spans="1:23" ht="45">
+    <row r="430" spans="1:23" ht="45" hidden="1">
       <c r="A430" s="3" t="s">
         <v>2333</v>
       </c>
@@ -61956,7 +61988,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="432" spans="1:23" ht="30">
+    <row r="432" spans="1:23" ht="30" hidden="1">
       <c r="A432" s="3" t="s">
         <v>2333</v>
       </c>
@@ -62098,7 +62130,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="434" spans="1:23" ht="30">
+    <row r="434" spans="1:23" ht="30" hidden="1">
       <c r="A434" s="3" t="s">
         <v>2333</v>
       </c>
@@ -62240,7 +62272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="436" spans="1:23" ht="30">
+    <row r="436" spans="1:23" ht="30" hidden="1">
       <c r="A436" s="3" t="s">
         <v>2333</v>
       </c>
@@ -62453,7 +62485,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="439" spans="1:23">
+    <row r="439" spans="1:23" hidden="1">
       <c r="A439" s="4" t="s">
         <v>2410</v>
       </c>
@@ -62524,7 +62556,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="440" spans="1:23" ht="30">
+    <row r="440" spans="1:23" ht="30" hidden="1">
       <c r="A440" s="4" t="s">
         <v>2410</v>
       </c>
@@ -62808,7 +62840,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="444" spans="1:23" ht="45">
+    <row r="444" spans="1:23" ht="45" hidden="1">
       <c r="A444" s="4" t="s">
         <v>2410</v>
       </c>
@@ -62950,7 +62982,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="446" spans="1:23" ht="30">
+    <row r="446" spans="1:23" ht="30" hidden="1">
       <c r="A446" s="4" t="s">
         <v>2410</v>
       </c>
@@ -63092,7 +63124,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="448" spans="1:23" ht="30">
+    <row r="448" spans="1:23" ht="30" hidden="1">
       <c r="A448" s="4" t="s">
         <v>2410</v>
       </c>
@@ -63305,7 +63337,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="451" spans="1:23" ht="30">
+    <row r="451" spans="1:23" ht="30" hidden="1">
       <c r="A451" s="3" t="s">
         <v>3655</v>
       </c>
@@ -63374,7 +63406,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="452" spans="1:23" ht="30">
+    <row r="452" spans="1:23" ht="30" hidden="1">
       <c r="A452" s="3" t="s">
         <v>3655</v>
       </c>
@@ -63443,7 +63475,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="453" spans="1:23" ht="30">
+    <row r="453" spans="1:23" ht="30" hidden="1">
       <c r="A453" s="3" t="s">
         <v>3655</v>
       </c>
@@ -63717,7 +63749,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="457" spans="1:23" ht="30">
+    <row r="457" spans="1:23" ht="30" hidden="1">
       <c r="A457" s="3" t="s">
         <v>3648</v>
       </c>
@@ -64129,7 +64161,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="463" spans="1:23" ht="30">
+    <row r="463" spans="1:23" ht="30" hidden="1">
       <c r="A463" s="4" t="s">
         <v>3955</v>
       </c>
@@ -64197,7 +64229,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="464" spans="1:23" ht="30">
+    <row r="464" spans="1:23" ht="30" hidden="1">
       <c r="A464" s="4" t="s">
         <v>3955</v>
       </c>
@@ -64469,7 +64501,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="468" spans="1:23" ht="30">
+    <row r="468" spans="1:23" ht="30" hidden="1">
       <c r="A468" s="4" t="s">
         <v>3955</v>
       </c>
@@ -64729,7 +64761,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="472" spans="1:23" ht="30">
+    <row r="472" spans="1:23" ht="30" hidden="1">
       <c r="A472" s="4" t="s">
         <v>3955</v>
       </c>
@@ -64862,7 +64894,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="474" spans="1:23" ht="30">
+    <row r="474" spans="1:23" ht="30" hidden="1">
       <c r="A474" s="4" t="s">
         <v>3955</v>
       </c>
@@ -64995,7 +65027,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="476" spans="1:23" ht="30">
+    <row r="476" spans="1:23" ht="30" hidden="1">
       <c r="A476" s="4" t="s">
         <v>3955</v>
       </c>
@@ -65199,7 +65231,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="479" spans="1:23" ht="30">
+    <row r="479" spans="1:23" ht="30" hidden="1">
       <c r="A479" s="4" t="s">
         <v>3954</v>
       </c>
@@ -65267,7 +65299,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="480" spans="1:23" ht="30">
+    <row r="480" spans="1:23" ht="30" hidden="1">
       <c r="A480" s="4" t="s">
         <v>3954</v>
       </c>
@@ -65335,7 +65367,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="481" spans="1:23" ht="30">
+    <row r="481" spans="1:23" ht="30" hidden="1">
       <c r="A481" s="4" t="s">
         <v>3954</v>
       </c>
@@ -65403,7 +65435,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="482" spans="1:23">
+    <row r="482" spans="1:23" hidden="1">
       <c r="A482" s="4" t="s">
         <v>3954</v>
       </c>
@@ -65539,7 +65571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="484" spans="1:23" ht="30">
+    <row r="484" spans="1:23" ht="30" hidden="1">
       <c r="A484" s="4" t="s">
         <v>3954</v>
       </c>
@@ -65740,7 +65772,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="487" spans="1:23" ht="30">
+    <row r="487" spans="1:23" ht="30" hidden="1">
       <c r="A487" s="4" t="s">
         <v>3954</v>
       </c>
@@ -66059,7 +66091,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="492" spans="1:23" ht="30">
+    <row r="492" spans="1:23" ht="30" hidden="1">
       <c r="A492" s="4" t="s">
         <v>3954</v>
       </c>
@@ -66192,7 +66224,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="494" spans="1:23" ht="30">
+    <row r="494" spans="1:23" ht="30" hidden="1">
       <c r="A494" s="4" t="s">
         <v>3954</v>
       </c>
@@ -66396,7 +66428,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="497" spans="1:23" ht="30">
+    <row r="497" spans="1:23" ht="30" hidden="1">
       <c r="A497" s="4" t="s">
         <v>4120</v>
       </c>
@@ -66804,7 +66836,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="503" spans="1:23" ht="30">
+    <row r="503" spans="1:23" ht="30" hidden="1">
       <c r="A503" s="4" t="s">
         <v>4120</v>
       </c>
@@ -66937,7 +66969,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="505" spans="1:23" ht="30">
+    <row r="505" spans="1:23" ht="30" hidden="1">
       <c r="A505" s="4" t="s">
         <v>4120</v>
       </c>
@@ -67070,7 +67102,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="507" spans="1:23" ht="30">
+    <row r="507" spans="1:23" ht="30" hidden="1">
       <c r="A507" s="4" t="s">
         <v>4120</v>
       </c>
@@ -67274,7 +67306,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="510" spans="1:23" ht="30">
+    <row r="510" spans="1:23" ht="30" hidden="1">
       <c r="A510" s="4" t="s">
         <v>3950</v>
       </c>
@@ -67342,7 +67374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="511" spans="1:23" ht="30">
+    <row r="511" spans="1:23" ht="30" hidden="1">
       <c r="A511" s="4" t="s">
         <v>3950</v>
       </c>
@@ -67410,7 +67442,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="512" spans="1:23" ht="30">
+    <row r="512" spans="1:23" ht="30" hidden="1">
       <c r="A512" s="4" t="s">
         <v>3950</v>
       </c>
@@ -67546,7 +67578,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="514" spans="1:23" ht="30">
+    <row r="514" spans="1:23" ht="30" hidden="1">
       <c r="A514" s="4" t="s">
         <v>3950</v>
       </c>
@@ -67679,7 +67711,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="516" spans="1:23" ht="30">
+    <row r="516" spans="1:23" ht="30" hidden="1">
       <c r="A516" s="4" t="s">
         <v>3950</v>
       </c>
@@ -67812,7 +67844,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="518" spans="1:23" ht="30">
+    <row r="518" spans="1:23" ht="30" hidden="1">
       <c r="A518" s="4" t="s">
         <v>3950</v>
       </c>
@@ -69365,7 +69397,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="540" spans="1:23" ht="30">
+    <row r="540" spans="1:23" ht="30" hidden="1">
       <c r="A540" s="4" t="s">
         <v>4290</v>
       </c>
@@ -69436,7 +69468,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="541" spans="1:23" ht="30">
+    <row r="541" spans="1:23" ht="30" hidden="1">
       <c r="A541" s="4" t="s">
         <v>4290</v>
       </c>
@@ -70217,7 +70249,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="552" spans="1:23" ht="30">
+    <row r="552" spans="1:23" ht="30" hidden="1">
       <c r="A552" s="4" t="s">
         <v>4290</v>
       </c>
@@ -70359,7 +70391,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="554" spans="1:23" ht="30">
+    <row r="554" spans="1:23" ht="30" hidden="1">
       <c r="A554" s="4" t="s">
         <v>4290</v>
       </c>
@@ -70501,7 +70533,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="556" spans="1:23" ht="30">
+    <row r="556" spans="1:23" ht="30" hidden="1">
       <c r="A556" s="4" t="s">
         <v>4290</v>
       </c>
@@ -70714,7 +70746,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="559" spans="1:23" ht="30">
+    <row r="559" spans="1:23" ht="30" hidden="1">
       <c r="A559" s="4" t="s">
         <v>4325</v>
       </c>
@@ -70785,7 +70817,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="560" spans="1:23" ht="30">
+    <row r="560" spans="1:23" ht="30" hidden="1">
       <c r="A560" s="4" t="s">
         <v>4325</v>
       </c>
@@ -70927,7 +70959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="562" spans="1:23" ht="60">
+    <row r="562" spans="1:23" ht="60" hidden="1">
       <c r="A562" s="4" t="s">
         <v>4325</v>
       </c>
@@ -71140,7 +71172,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="565" spans="1:23" ht="45">
+    <row r="565" spans="1:23" ht="45" hidden="1">
       <c r="A565" s="4" t="s">
         <v>4325</v>
       </c>
@@ -71282,7 +71314,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="567" spans="1:23" ht="45">
+    <row r="567" spans="1:23" ht="45" hidden="1">
       <c r="A567" s="4" t="s">
         <v>4325</v>
       </c>
@@ -71353,7 +71385,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="568" spans="1:23" ht="30">
+    <row r="568" spans="1:23" ht="30" hidden="1">
       <c r="A568" s="4" t="s">
         <v>4325</v>
       </c>
@@ -71495,7 +71527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="570" spans="1:23" ht="30">
+    <row r="570" spans="1:23" ht="30" hidden="1">
       <c r="A570" s="4" t="s">
         <v>4325</v>
       </c>
@@ -71637,7 +71669,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="572" spans="1:23" ht="30">
+    <row r="572" spans="1:23" ht="30" hidden="1">
       <c r="A572" s="4" t="s">
         <v>4325</v>
       </c>
@@ -71850,7 +71882,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="575" spans="1:23" ht="30">
+    <row r="575" spans="1:23" ht="30" hidden="1">
       <c r="A575" s="4" t="s">
         <v>4332</v>
       </c>
@@ -71921,7 +71953,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="576" spans="1:23" ht="30">
+    <row r="576" spans="1:23" ht="30" hidden="1">
       <c r="A576" s="4" t="s">
         <v>4332</v>
       </c>
@@ -71992,7 +72024,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="577" spans="1:23" ht="45">
+    <row r="577" spans="1:23" ht="45" hidden="1">
       <c r="A577" s="4" t="s">
         <v>4332</v>
       </c>
@@ -72134,7 +72166,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="579" spans="1:23" ht="30">
+    <row r="579" spans="1:23" ht="30" hidden="1">
       <c r="A579" s="4" t="s">
         <v>4332</v>
       </c>
@@ -72205,7 +72237,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="580" spans="1:23" ht="30">
+    <row r="580" spans="1:23" ht="30" hidden="1">
       <c r="A580" s="4" t="s">
         <v>4332</v>
       </c>
@@ -72276,7 +72308,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="581" spans="1:23" ht="45">
+    <row r="581" spans="1:23" ht="45" hidden="1">
       <c r="A581" s="4" t="s">
         <v>4332</v>
       </c>
@@ -72489,7 +72521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="584" spans="1:23" ht="30">
+    <row r="584" spans="1:23" ht="30" hidden="1">
       <c r="A584" s="4" t="s">
         <v>4332</v>
       </c>
@@ -72702,7 +72734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="587" spans="1:23" ht="45">
+    <row r="587" spans="1:23" ht="45" hidden="1">
       <c r="A587" s="4" t="s">
         <v>4332</v>
       </c>
@@ -72844,7 +72876,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="589" spans="1:23" ht="45">
+    <row r="589" spans="1:23" ht="45" hidden="1">
       <c r="A589" s="4" t="s">
         <v>4480</v>
       </c>
@@ -72915,7 +72947,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="590" spans="1:23" ht="45">
+    <row r="590" spans="1:23" ht="45" hidden="1">
       <c r="A590" s="4" t="s">
         <v>4480</v>
       </c>
@@ -72986,7 +73018,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="591" spans="1:23" ht="45">
+    <row r="591" spans="1:23" ht="45" hidden="1">
       <c r="A591" s="4" t="s">
         <v>4480</v>
       </c>
@@ -73057,7 +73089,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="592" spans="1:23" ht="30">
+    <row r="592" spans="1:23" ht="30" hidden="1">
       <c r="A592" s="4" t="s">
         <v>4480</v>
       </c>
@@ -73128,7 +73160,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="593" spans="1:23" ht="30">
+    <row r="593" spans="1:23" ht="30" hidden="1">
       <c r="A593" s="4" t="s">
         <v>4480</v>
       </c>
@@ -73199,7 +73231,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="594" spans="1:23" ht="45">
+    <row r="594" spans="1:23" ht="45" hidden="1">
       <c r="A594" s="4" t="s">
         <v>4480</v>
       </c>
@@ -73412,7 +73444,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="597" spans="1:23" ht="30">
+    <row r="597" spans="1:23" ht="30" hidden="1">
       <c r="A597" s="4" t="s">
         <v>4480</v>
       </c>
@@ -73554,7 +73586,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="599" spans="1:23" ht="30">
+    <row r="599" spans="1:23" ht="30" hidden="1">
       <c r="A599" s="4" t="s">
         <v>4526</v>
       </c>
@@ -73619,7 +73651,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="600" spans="1:23" ht="30">
+    <row r="600" spans="1:23" ht="30" hidden="1">
       <c r="A600" s="4" t="s">
         <v>4526</v>
       </c>
@@ -73752,7 +73784,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="602" spans="1:23" ht="30">
+    <row r="602" spans="1:23" ht="30" hidden="1">
       <c r="A602" s="4" t="s">
         <v>4526</v>
       </c>
@@ -73944,7 +73976,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="605" spans="1:23" ht="30">
+    <row r="605" spans="1:23" ht="30" hidden="1">
       <c r="A605" s="4" t="s">
         <v>4526</v>
       </c>
@@ -74074,7 +74106,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="607" spans="1:23" ht="30">
+    <row r="607" spans="1:23" ht="30" hidden="1">
       <c r="A607" s="4" t="s">
         <v>4526</v>
       </c>
@@ -74204,7 +74236,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="609" spans="1:23" ht="30">
+    <row r="609" spans="1:23" ht="30" hidden="1">
       <c r="A609" s="4" t="s">
         <v>4526</v>
       </c>
@@ -74404,6 +74436,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:W611" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Benefit Usage Rule"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="4">
       <filters>
         <filter val="Identifier"/>
@@ -76058,7 +76095,7 @@
       </c>
       <c r="I49" s="3"/>
     </row>
-    <row r="50" spans="1:9" ht="30">
+    <row r="50" spans="1:9">
       <c r="A50" s="3" t="s">
         <v>516</v>
       </c>
@@ -76716,7 +76753,7 @@
       </c>
       <c r="I73" s="3"/>
     </row>
-    <row r="74" spans="1:9" ht="30">
+    <row r="74" spans="1:9">
       <c r="A74" s="3" t="s">
         <v>94</v>
       </c>
@@ -76770,7 +76807,7 @@
       </c>
       <c r="I75" s="3"/>
     </row>
-    <row r="76" spans="1:9" ht="30">
+    <row r="76" spans="1:9">
       <c r="A76" s="3" t="s">
         <v>94</v>
       </c>
@@ -76882,7 +76919,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="45">
+    <row r="80" spans="1:9" ht="30">
       <c r="A80" s="3" t="s">
         <v>1689</v>
       </c>
@@ -77143,7 +77180,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="30">
+    <row r="89" spans="1:9">
       <c r="A89" s="3" t="s">
         <v>1689</v>
       </c>

</xml_diff>

<commit_message>
Customer experience preview screen impl server
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CDBDB1-6377-4522-9E8C-56B83BBCD2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A27D54-4033-45E7-9672-DD73764726ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="11" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="11" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19517" uniqueCount="4931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19523" uniqueCount="4935">
   <si>
     <t>Domain</t>
   </si>
@@ -14837,13 +14837,25 @@
   </si>
   <si>
     <t>BENEFIT_USAGE_RULE</t>
+  </si>
+  <si>
+    <t>CUSTOMER_EXPERIENCE</t>
+  </si>
+  <si>
+    <t>DRAFT, PUBLISHED, INACTIVE, RETIRED</t>
+  </si>
+  <si>
+    <t>CUSTOMER_EXPERIENCE_RELEASE</t>
+  </si>
+  <si>
+    <t>PUBLISHED, ARCHIVED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -14884,6 +14896,13 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -14912,7 +14931,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -14976,6 +14995,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16528,7 +16550,7 @@
         <v>1130</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="45">
+    <row r="22" spans="1:17" ht="30">
       <c r="A22" s="4" t="s">
         <v>1164</v>
       </c>
@@ -19610,7 +19632,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7B29B1-81FD-48F8-9727-C5470F35164D}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" style="4" bestFit="1" customWidth="1"/>
@@ -20010,6 +20032,34 @@
       </c>
       <c r="D28" t="s">
         <v>2235</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="23">
+        <v>28</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>2333</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>4931</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>4932</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="23">
+        <v>29</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>4526</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>4933</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>4934</v>
       </c>
     </row>
   </sheetData>
@@ -37359,7 +37409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="45" hidden="1">
+    <row r="79" spans="1:23" ht="30" hidden="1">
       <c r="A79" s="4" t="s">
         <v>10</v>
       </c>
@@ -37430,7 +37480,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="45" hidden="1">
+    <row r="80" spans="1:23" ht="30" hidden="1">
       <c r="A80" s="4" t="s">
         <v>10</v>
       </c>

</xml_diff>